<commit_message>
safeguards questions selectors updated
</commit_message>
<xml_diff>
--- a/src/data/output/cp_output.xlsx
+++ b/src/data/output/cp_output.xlsx
@@ -543,27 +543,27 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>0100465</t>
+          <t>0100498</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>57525.00</t>
+          <t>55992.50</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>2682.58</t>
+          <t>2677.98</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>2876.26</t>
+          <t>2799.63</t>
         </is>
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>63083.84</t>
+          <t>61470.11</t>
         </is>
       </c>
     </row>
@@ -575,27 +575,27 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>0100353</t>
+          <t>0100509</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>11610.91</t>
+          <t>11115.50</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>815.00</t>
+          <t>810.00</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>565.37</t>
+          <t>542.61</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>12991.28</t>
+          <t>12468.11</t>
         </is>
       </c>
     </row>
@@ -607,27 +607,27 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>0100356</t>
+          <t>0100773</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>32856.94</t>
+          <t>31239.00</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>1525.00</t>
+          <t>1500.00</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>1031.46</t>
+          <t>982.17</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>35413.40</t>
+          <t>33721.17</t>
         </is>
       </c>
     </row>
@@ -639,27 +639,27 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>0100362</t>
+          <t>0100516</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>26168.96</t>
+          <t>25413.50</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>1520.00</t>
+          <t>1525.00</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>623.00</t>
+          <t>606.12</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>28321.65</t>
+          <t>27554.05</t>
         </is>
       </c>
     </row>
@@ -671,27 +671,27 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>0100347</t>
+          <t>0100497</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>16115.51</t>
+          <t>15585.00</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>1125.00</t>
+          <t>1090.95</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>483.47</t>
+          <t>467.55</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>17723.98</t>
+          <t>17143.50</t>
         </is>
       </c>
     </row>
@@ -703,27 +703,27 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>0100350</t>
+          <t>0100505</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>27755.90</t>
+          <t>26990.00</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>1855.00</t>
+          <t>1870.00</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>592.22</t>
+          <t>577.20</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>30203.12</t>
+          <t>29437.20</t>
         </is>
       </c>
     </row>
@@ -735,27 +735,27 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>0100354</t>
+          <t>0100510</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>14272.82</t>
+          <t>14573.50</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>642.82</t>
+          <t>658.72</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>713.64</t>
+          <t>728.68</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>15629.28</t>
+          <t>15960.90</t>
         </is>
       </c>
     </row>
@@ -767,27 +767,27 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>0100358</t>
+          <t>0100514</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>46294.30</t>
+          <t>45698.50</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>4245.00</t>
+          <t>4310.00</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>2299.54</t>
+          <t>2275.39</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>52838.84</t>
+          <t>52283.89</t>
         </is>
       </c>
     </row>
@@ -799,27 +799,27 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>0100346</t>
+          <t>0100499</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>47741.04</t>
+          <t>48145.00</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>2860.00</t>
+          <t>2960.00</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>1518.03</t>
+          <t>1533.15</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>52119.07</t>
+          <t>52638.15</t>
         </is>
       </c>
     </row>
@@ -831,27 +831,27 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>0100355</t>
+          <t>0100512</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>36809.83</t>
+          <t>35492.50</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>2140.00</t>
+          <t>2125.00</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>1104.29</t>
+          <t>1064.78</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>40054.12</t>
+          <t>38682.28</t>
         </is>
       </c>
     </row>
@@ -863,27 +863,27 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>0100428</t>
+          <t>0100517</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>53526.18</t>
+          <t>50907.50</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>3580.58</t>
+          <t>3502.72</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>2676.31</t>
+          <t>2545.38</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>59783.07</t>
+          <t>56955.60</t>
         </is>
       </c>
     </row>
@@ -895,27 +895,27 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>0100366</t>
+          <t>0100798</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>34116.51</t>
+          <t>33959.50</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>1205.00</t>
+          <t>1220.00</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>1607.12</t>
+          <t>1600.67</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>36928.63</t>
+          <t>36780.17</t>
         </is>
       </c>
     </row>
@@ -927,27 +927,27 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>0100345</t>
+          <t>0100771</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>12318.58</t>
+          <t>12029.50</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>1220.00</t>
+          <t>1225.00</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>406.16</t>
+          <t>397.64</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>13944.74</t>
+          <t>13652.14</t>
         </is>
       </c>
     </row>
@@ -959,27 +959,27 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>0100349</t>
+          <t>0100501</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>13626.08</t>
+          <t>12727.50</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>930.00</t>
+          <t>910.00</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>408.78</t>
+          <t>381.83</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>14964.86</t>
+          <t>14019.33</t>
         </is>
       </c>
     </row>
@@ -991,27 +991,27 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>0100351</t>
+          <t>0100504</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>32504.59</t>
+          <t>31072.50</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>707.51</t>
+          <t>703.22</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>1625.23</t>
+          <t>1553.63</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>34837.33</t>
+          <t>33329.35</t>
         </is>
       </c>
     </row>
@@ -1023,27 +1023,27 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>0100357</t>
+          <t>0100508</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>21342.46</t>
+          <t>19537.50</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>1475.00</t>
+          <t>1430.00</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>1038.20</t>
+          <t>954.02</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>23855.66</t>
+          <t>21921.52</t>
         </is>
       </c>
     </row>
@@ -1055,27 +1055,27 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>0100434</t>
+          <t>0100515</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>8336.08</t>
+          <t>8237.00</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>675.00</t>
+          <t>680.00</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>270.33</t>
+          <t>267.51</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>9281.41</t>
+          <t>9184.51</t>
         </is>
       </c>
     </row>
@@ -1087,27 +1087,27 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>0100363</t>
+          <t>0100774</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>13560.40</t>
+          <t>12756.00</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>1130.00</t>
+          <t>1120.00</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>330.54</t>
+          <t>312.21</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>15026.08</t>
+          <t>14193.07</t>
         </is>
       </c>
     </row>
@@ -1119,27 +1119,27 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>0100364</t>
+          <t>0100524</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>20869.02</t>
+          <t>20736.50</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>555.00</t>
+          <t>560.00</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>626.07</t>
+          <t>622.10</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>22050.09</t>
+          <t>21918.60</t>
         </is>
       </c>
     </row>
@@ -1151,27 +1151,27 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>0100382</t>
+          <t>0100531</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>41283.49</t>
+          <t>41080.00</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>3760.00</t>
+          <t>3860.00</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>1238.50</t>
+          <t>1232.40</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>46281.99</t>
+          <t>46172.40</t>
         </is>
       </c>
     </row>
@@ -1183,27 +1183,27 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>0100390</t>
+          <t>0100769</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>59103.12</t>
+          <t>60469.00</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>1532.31</t>
+          <t>1591.41</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>2955.16</t>
+          <t>3023.45</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>63590.59</t>
+          <t>65083.86</t>
         </is>
       </c>
     </row>
@@ -1215,12 +1215,12 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>0100429</t>
+          <t>0100526</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>41403.05</t>
+          <t>39066.50</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
@@ -1230,12 +1230,12 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>1252.59</t>
+          <t>1182.50</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>43005.64</t>
+          <t>40599.00</t>
         </is>
       </c>
     </row>
@@ -1247,27 +1247,27 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>0100389</t>
+          <t>0100542</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>28180.90</t>
+          <t>29071.50</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>2165.00</t>
+          <t>2290.00</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>682.78</t>
+          <t>705.63</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>31039.30</t>
+          <t>32078.11</t>
         </is>
       </c>
     </row>
@@ -1279,27 +1279,27 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>0100383</t>
+          <t>0100551</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>27017.95</t>
+          <t>25330.00</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>1630.00</t>
+          <t>1590.00</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>572.96</t>
+          <t>538.40</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>29220.91</t>
+          <t>27458.40</t>
         </is>
       </c>
     </row>
@@ -1311,27 +1311,27 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>0100433</t>
+          <t>0100770</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>32399.24</t>
+          <t>33055.50</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>3255.00</t>
+          <t>3380.00</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>971.98</t>
+          <t>991.67</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>36626.22</t>
+          <t>37427.17</t>
         </is>
       </c>
     </row>
@@ -1343,27 +1343,27 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>0100392</t>
+          <t>0100520</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>38187.86</t>
+          <t>36392.50</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>2830.00</t>
+          <t>2820.00</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>1866.31</t>
+          <t>1784.17</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>42884.17</t>
+          <t>40996.67</t>
         </is>
       </c>
     </row>
@@ -1375,27 +1375,27 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>0100394</t>
+          <t>0100777</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>60898.93</t>
+          <t>62316.50</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>3215.00</t>
+          <t>3370.00</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>1826.97</t>
+          <t>1869.50</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>65940.90</t>
+          <t>67556.00</t>
         </is>
       </c>
     </row>
@@ -1407,27 +1407,27 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>0100401</t>
+          <t>0100549</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>20675.14</t>
+          <t>20774.00</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>1855.00</t>
+          <t>1905.00</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>450.60</t>
+          <t>453.58</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>22980.74</t>
+          <t>23132.58</t>
         </is>
       </c>
     </row>
@@ -1439,27 +1439,27 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>0100391</t>
+          <t>0100772</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>49446.33</t>
+          <t>47937.00</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>2840.00</t>
+          <t>2830.00</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>1483.39</t>
+          <t>1438.11</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>53769.72</t>
+          <t>52205.11</t>
         </is>
       </c>
     </row>
@@ -1471,27 +1471,27 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>0100396</t>
+          <t>0100538</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>33916.46</t>
+          <t>32778.00</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>2756.75</t>
+          <t>2743.33</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>1695.82</t>
+          <t>1638.90</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>38369.03</t>
+          <t>37160.23</t>
         </is>
       </c>
     </row>
@@ -1503,27 +1503,27 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>0100430</t>
+          <t>0100546</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>30081.04</t>
+          <t>29541.50</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>1170.00</t>
+          <t>1190.00</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>1421.92</t>
+          <t>1398.28</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>32672.96</t>
+          <t>32129.78</t>
         </is>
       </c>
     </row>
@@ -1533,11 +1533,31 @@
           <t>TS-032</t>
         </is>
       </c>
-      <c r="B33" s="5" t="n"/>
-      <c r="C33" s="5" t="n"/>
-      <c r="D33" s="5" t="n"/>
-      <c r="E33" s="5" t="n"/>
-      <c r="F33" s="5" t="n"/>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>0100604</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>26894.50</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>1095.00</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>629.76</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>28629.06</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="15" customHeight="1">
       <c r="A34" s="7" t="inlineStr">
@@ -1547,27 +1567,27 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>0100400</t>
+          <t>0100617</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>25298.11</t>
+          <t>24567.50</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>1770.87</t>
+          <t>1719.73</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>758.94</t>
+          <t>737.03</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>27827.92</t>
+          <t>27024.26</t>
         </is>
       </c>
     </row>
@@ -1579,27 +1599,27 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>0100405</t>
+          <t>0100601</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>25838.86</t>
+          <t>25489.00</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>930.00</t>
+          <t>935.00</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>535.38</t>
+          <t>528.48</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>27304.24</t>
+          <t>26952.48</t>
         </is>
       </c>
     </row>
@@ -1611,27 +1631,27 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>0100404</t>
+          <t>0100780</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>74732.89</t>
+          <t>66731.50</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>7760.00</t>
+          <t>7145.00</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>2241.99</t>
+          <t>2001.95</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>84734.88</t>
+          <t>75878.45</t>
         </is>
       </c>
     </row>
@@ -1643,27 +1663,27 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>0100427</t>
+          <t>0100602</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>48366.90</t>
+          <t>50247.50</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>795.10</t>
+          <t>800.74</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>2418.35</t>
+          <t>2512.38</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>51580.35</t>
+          <t>53560.62</t>
         </is>
       </c>
     </row>
@@ -1675,27 +1695,27 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>0100435</t>
+          <t>0100618</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>27225.84</t>
+          <t>25521.50</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>1905.81</t>
+          <t>1786.51</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>816.78</t>
+          <t>765.65</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>29948.43</t>
+          <t>28073.66</t>
         </is>
       </c>
     </row>
@@ -1707,27 +1727,27 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>0100440</t>
+          <t>0100603</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>23303.86</t>
+          <t>23926.00</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>705.00</t>
+          <t>730.00</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>480.18</t>
+          <t>493.12</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>24489.04</t>
+          <t>25149.12</t>
         </is>
       </c>
     </row>
@@ -1739,27 +1759,27 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>0100411</t>
+          <t>0100775</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>24491.59</t>
+          <t>24906.50</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>1540.00</t>
+          <t>1590.00</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>734.75</t>
+          <t>747.20</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>26766.34</t>
+          <t>27243.70</t>
         </is>
       </c>
     </row>
@@ -1771,27 +1791,27 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>0100410</t>
+          <t>0100611</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>32344.34</t>
+          <t>30744.50</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>3432.03</t>
+          <t>3367.23</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>1617.22</t>
+          <t>1537.23</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>37393.59</t>
+          <t>35648.96</t>
         </is>
       </c>
     </row>
@@ -1803,27 +1823,27 @@
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>0100413</t>
+          <t>0100644</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>38915.80</t>
+          <t>35885.50</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>1300.00</t>
+          <t>1250.00</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>904.85</t>
+          <t>835.55</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>41134.72</t>
+          <t>37984.05</t>
         </is>
       </c>
     </row>
@@ -1835,27 +1855,27 @@
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>0100415</t>
+          <t>0100652</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>34096.99</t>
+          <t>34462.00</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>1935.00</t>
+          <t>2005.00</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>1022.91</t>
+          <t>1033.86</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>37054.90</t>
+          <t>37500.86</t>
         </is>
       </c>
     </row>
@@ -1867,27 +1887,27 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>0100417</t>
+          <t>0100643</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>43508.26</t>
+          <t>38721.00</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>975.00</t>
+          <t>940.00</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>889.67</t>
+          <t>793.22</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>45372.93</t>
+          <t>40454.22</t>
         </is>
       </c>
     </row>
@@ -1899,27 +1919,27 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>0100416</t>
+          <t>0100657</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>32157.66</t>
+          <t>31393.00</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>2440.00</t>
+          <t>2455.00</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>964.73</t>
+          <t>941.79</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>35562.39</t>
+          <t>34789.79</t>
         </is>
       </c>
     </row>
@@ -1931,27 +1951,27 @@
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>0100419</t>
+          <t>0100797</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>70538.38</t>
+          <t>72066.50</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>6361.62</t>
+          <t>6646.20</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>3526.92</t>
+          <t>3603.33</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>80426.92</t>
+          <t>82316.03</t>
         </is>
       </c>
     </row>
@@ -1963,27 +1983,27 @@
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>0100420</t>
+          <t>0100656</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>53796.84</t>
+          <t>50891.00</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>2280.00</t>
+          <t>2235.00</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>2551.50</t>
+          <t>2417.23</t>
         </is>
       </c>
       <c r="F47" s="4" t="inlineStr">
         <is>
-          <t>58628.34</t>
+          <t>55543.23</t>
         </is>
       </c>
     </row>
@@ -1995,27 +2015,27 @@
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>0100422</t>
+          <t>0100646</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>65723.17</t>
+          <t>61048.50</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>6430.00</t>
+          <t>6145.00</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>1623.45</t>
+          <t>1511.85</t>
         </is>
       </c>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t>73801.88</t>
+          <t>68728.87</t>
         </is>
       </c>
     </row>
@@ -2027,27 +2047,27 @@
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>0100424</t>
+          <t>0100658</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>11289.35</t>
+          <t>11037.50</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>790.25</t>
+          <t>772.63</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>338.68</t>
+          <t>331.13</t>
         </is>
       </c>
       <c r="F49" s="4" t="inlineStr">
         <is>
-          <t>12418.28</t>
+          <t>12141.26</t>
         </is>
       </c>
     </row>
@@ -2059,27 +2079,27 @@
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>0100425</t>
+          <t>0100778</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>65784.51</t>
+          <t>63999.00</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>1535.00</t>
+          <t>1530.00</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>1346.39</t>
+          <t>1310.58</t>
         </is>
       </c>
       <c r="F50" s="4" t="inlineStr">
         <is>
-          <t>68665.90</t>
+          <t>66839.58</t>
         </is>
       </c>
     </row>
@@ -2091,27 +2111,27 @@
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>0100426</t>
+          <t>0100779</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>49557.29</t>
+          <t>50484.00</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>2090.00</t>
+          <t>2165.00</t>
         </is>
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t>1549.42</t>
+          <t>1579.47</t>
         </is>
       </c>
       <c r="F51" s="4" t="inlineStr">
         <is>
-          <t>53196.71</t>
+          <t>54228.47</t>
         </is>
       </c>
     </row>
@@ -2123,27 +2143,27 @@
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>0100441</t>
+          <t>0100781</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>28842.73</t>
+          <t>27967.50</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>2480.00</t>
+          <t>2490.00</t>
         </is>
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>704.76</t>
+          <t>685.29</t>
         </is>
       </c>
       <c r="F52" s="4" t="inlineStr">
         <is>
-          <t>32038.45</t>
+          <t>31153.45</t>
         </is>
       </c>
     </row>
@@ -2153,11 +2173,31 @@
           <t>TS-052</t>
         </is>
       </c>
-      <c r="B53" s="4" t="n"/>
-      <c r="C53" s="4" t="n"/>
-      <c r="D53" s="4" t="n"/>
-      <c r="E53" s="4" t="n"/>
-      <c r="F53" s="4" t="n"/>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>0100783</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>10415.00</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t>205.00</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="inlineStr">
+        <is>
+          <t>312.45</t>
+        </is>
+      </c>
+      <c r="F53" s="4" t="inlineStr">
+        <is>
+          <t>10932.45</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="15" customHeight="1">
       <c r="A54" s="7" t="inlineStr">
@@ -2167,27 +2207,27 @@
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>0100438</t>
+          <t>0100799</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>10612.66</t>
+          <t>10550.50</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>560.00</t>
+          <t>575.00</t>
         </is>
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>508.36</t>
+          <t>506.21</t>
         </is>
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>11681.02</t>
+          <t>11631.71</t>
         </is>
       </c>
     </row>
@@ -2199,27 +2239,27 @@
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>0100439</t>
+          <t>0100667</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>16308.38</t>
+          <t>15993.50</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>1045.00</t>
+          <t>1050.00</t>
         </is>
       </c>
       <c r="E55" s="4" t="inlineStr">
         <is>
-          <t>520.60</t>
+          <t>511.31</t>
         </is>
       </c>
       <c r="F55" s="4" t="inlineStr">
         <is>
-          <t>17873.98</t>
+          <t>17554.81</t>
         </is>
       </c>
     </row>
@@ -2231,27 +2271,27 @@
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t>0100442</t>
+          <t>0100786</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>57626.36</t>
+          <t>50501.00</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>2605.00</t>
+          <t>2420.00</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
-          <t>1355.21</t>
+          <t>1190.72</t>
         </is>
       </c>
       <c r="F56" s="4" t="inlineStr">
         <is>
-          <t>61607.65</t>
+          <t>54130.24</t>
         </is>
       </c>
     </row>
@@ -2263,27 +2303,27 @@
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>0100443</t>
+          <t>0100782</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>21507.50</t>
+          <t>20202.50</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t>1290.00</t>
+          <t>1265.00</t>
         </is>
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t>645.23</t>
+          <t>606.08</t>
         </is>
       </c>
       <c r="F57" s="4" t="inlineStr">
         <is>
-          <t>23442.73</t>
+          <t>22073.58</t>
         </is>
       </c>
     </row>
@@ -2295,27 +2335,27 @@
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>0100444</t>
+          <t>0100789</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>38495.06</t>
+          <t>39377.00</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>1605.00</t>
+          <t>1680.00</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t>802.00</t>
+          <t>821.14</t>
         </is>
       </c>
       <c r="F58" s="4" t="inlineStr">
         <is>
-          <t>40902.06</t>
+          <t>41878.14</t>
         </is>
       </c>
     </row>
@@ -2327,27 +2367,27 @@
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>0100445</t>
+          <t>0100785</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>64540.84</t>
+          <t>64553.50</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>3163.62</t>
+          <t>3228.66</t>
         </is>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
-          <t>3227.04</t>
+          <t>3227.68</t>
         </is>
       </c>
       <c r="F59" s="4" t="inlineStr">
         <is>
-          <t>70931.50</t>
+          <t>71009.84</t>
         </is>
       </c>
     </row>
@@ -2359,27 +2399,27 @@
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>0100447</t>
+          <t>0100713</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>33150.36</t>
+          <t>31854.50</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>2165.00</t>
+          <t>2145.00</t>
         </is>
       </c>
       <c r="E60" s="4" t="inlineStr">
         <is>
-          <t>1606.85</t>
+          <t>1546.98</t>
         </is>
       </c>
       <c r="F60" s="4" t="inlineStr">
         <is>
-          <t>36922.21</t>
+          <t>35546.48</t>
         </is>
       </c>
     </row>
@@ -2391,27 +2431,27 @@
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>0100446</t>
+          <t>0100788</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>23317.82</t>
+          <t>21765.00</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>1575.00</t>
+          <t>1540.00</t>
         </is>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>746.78</t>
+          <t>699.15</t>
         </is>
       </c>
       <c r="F61" s="4" t="inlineStr">
         <is>
-          <t>25639.60</t>
+          <t>24004.15</t>
         </is>
       </c>
     </row>
@@ -2423,27 +2463,27 @@
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>0100452</t>
+          <t>0100711</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>24687.54</t>
+          <t>23501.00</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>2310.00</t>
+          <t>2255.00</t>
         </is>
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
-          <t>740.63</t>
+          <t>705.03</t>
         </is>
       </c>
       <c r="F62" s="4" t="inlineStr">
         <is>
-          <t>27738.17</t>
+          <t>26461.03</t>
         </is>
       </c>
     </row>
@@ -2455,27 +2495,27 @@
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>0100453</t>
+          <t>0100792</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>75905.03</t>
+          <t>73874.00</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>4387.72</t>
+          <t>4366.62</t>
         </is>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>3795.25</t>
+          <t>3693.70</t>
         </is>
       </c>
       <c r="F63" s="4" t="inlineStr">
         <is>
-          <t>84088.00</t>
+          <t>81934.32</t>
         </is>
       </c>
     </row>
@@ -2487,27 +2527,27 @@
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
-          <t>0100450</t>
+          <t>0100717</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>35926.07</t>
+          <t>37546.00</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t>1170.00</t>
+          <t>1215.00</t>
         </is>
       </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
-          <t>1687.87</t>
+          <t>1763.63</t>
         </is>
       </c>
       <c r="F64" s="4" t="inlineStr">
         <is>
-          <t>38783.94</t>
+          <t>40524.63</t>
         </is>
       </c>
     </row>
@@ -2519,27 +2559,27 @@
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>0100451</t>
+          <t>0100718</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>30213.70</t>
+          <t>30346.00</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t>3390.00</t>
+          <t>3485.00</t>
         </is>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>756.09</t>
+          <t>761.20</t>
         </is>
       </c>
       <c r="F65" s="4" t="inlineStr">
         <is>
-          <t>34371.55</t>
+          <t>34604.04</t>
         </is>
       </c>
     </row>
@@ -2551,27 +2591,27 @@
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>0100459</t>
+          <t>0100715</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>53422.66</t>
+          <t>53003.00</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
         <is>
-          <t>2030.00</t>
+          <t>2065.00</t>
         </is>
       </c>
       <c r="E66" s="4" t="inlineStr">
         <is>
-          <t>1602.68</t>
+          <t>1590.09</t>
         </is>
       </c>
       <c r="F66" s="4" t="inlineStr">
         <is>
-          <t>57055.34</t>
+          <t>56658.09</t>
         </is>
       </c>
     </row>
@@ -2583,27 +2623,27 @@
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>0100454</t>
+          <t>0100716</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>32596.29</t>
+          <t>32064.50</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>3242.79</t>
+          <t>3276.19</t>
         </is>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>1629.81</t>
+          <t>1603.23</t>
         </is>
       </c>
       <c r="F67" s="4" t="inlineStr">
         <is>
-          <t>37468.89</t>
+          <t>36943.92</t>
         </is>
       </c>
     </row>

</xml_diff>